<commit_message>
feat: complete Travel OS lifecycle and validation
</commit_message>
<xml_diff>
--- a/templates/TravelOS-Template.xlsx
+++ b/templates/TravelOS-Template.xlsx
@@ -2,10 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旅行概览" sheetId="1" r:id="R11f90b7b6fc64149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前行程" sheetId="2" r:id="Ra898c79a5af24757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策与协作" sheetId="3" r:id="R4944575411664995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="4" r:id="Rce7bd37146704a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="R1923f46351a44bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R57f2af995ad545fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="R3f382a0ca7ce463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="Re882fef17dff4f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R10c94c6a9c9a44f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="R0d82132e5d19404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="R5b4c9e3a47264ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R0f4a7277c3624dd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -62,14 +66,23 @@
     </x:fill>
   </x:fills>
   <x:borders count="10">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -78,19 +91,25 @@
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
@@ -100,6 +119,7 @@
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -114,25 +134,31 @@
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -144,20 +170,25 @@
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -224,13 +255,25 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -441,18 +484,20 @@
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>旅行概览</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
+        <x:v>Travel Overview</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
         <x:v>Trip ID</x:v>
       </x:c>
@@ -478,13 +523,19 @@
         <x:v>Active Version</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
+        <x:v>旅行阶段</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="J2" s="10" t="str">
+      <x:c r="K2" s="9" t="str">
+        <x:v>主时区</x:v>
+      </x:c>
+      <x:c r="L2" s="10" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="24" customHeight="1">
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
         <x:v>DEMO-001</x:v>
       </x:c>
@@ -494,29 +545,35 @@
       <x:c r="C3" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="D3" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="E3" s="17" t="n">
-        <x:v>47606</x:v>
+      <x:c r="D3" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="d">
+        <x:v>2030-05-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
+        <x:v>M-001</x:v>
       </x:c>
       <x:c r="H3" s="21" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
       <x:c r="I3" s="12" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="J3" s="13" t="str">
+        <x:v>行前规划</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="str">
         <x:v>本行仅为虚构示例，请替换</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="24" customHeight="1">
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="15" t="str"/>
       <x:c r="C4" s="15" t="str"/>
@@ -526,11 +583,16 @@
       <x:c r="G4" s="15" t="str"/>
       <x:c r="H4" s="22" t="str"/>
       <x:c r="I4" s="15" t="str"/>
-      <x:c r="J4" s="16" t="str"/>
+      <x:c r="J4" s="15" t="str"/>
+      <x:c r="K4" s="15" t="str"/>
+      <x:c r="L4" s="16" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I3:I4">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="I3:I100">
+      <x:formula1>"行前规划,旅行中,旅行后"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J3:J100">
       <x:formula1>"Draft,Active,Completed,Cancelled"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -542,164 +604,210 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>当前行程</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
+        <x:v>Daily Plan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
+        <x:v>项目ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
         <x:v>版本</x:v>
       </x:c>
-      <x:c r="B2" s="9" t="str">
+      <x:c r="C2" s="9" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>开始</x:v>
       </x:c>
-      <x:c r="D2" s="9" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>结束</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="str">
+      <x:c r="F2" s="9" t="str">
+        <x:v>时区</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
         <x:v>城市</x:v>
       </x:c>
-      <x:c r="F2" s="9" t="str">
+      <x:c r="H2" s="9" t="str">
         <x:v>活动</x:v>
       </x:c>
-      <x:c r="G2" s="9" t="str">
+      <x:c r="I2" s="9" t="str">
         <x:v>地点</x:v>
       </x:c>
-      <x:c r="H2" s="9" t="str">
+      <x:c r="J2" s="9" t="str">
         <x:v>交通</x:v>
       </x:c>
-      <x:c r="I2" s="9" t="str">
-        <x:v>预订状态</x:v>
-      </x:c>
-      <x:c r="J2" s="9" t="str">
+      <x:c r="K2" s="9" t="str">
+        <x:v>预订ID</x:v>
+      </x:c>
+      <x:c r="L2" s="9" t="str">
+        <x:v>执行状态</x:v>
+      </x:c>
+      <x:c r="M2" s="9" t="str">
         <x:v>费用</x:v>
       </x:c>
-      <x:c r="K2" s="9" t="str">
+      <x:c r="N2" s="9" t="str">
         <x:v>币种</x:v>
       </x:c>
-      <x:c r="L2" s="9" t="str">
+      <x:c r="O2" s="9" t="str">
         <x:v>来源</x:v>
       </x:c>
-      <x:c r="M2" s="10" t="str">
+      <x:c r="P2" s="9" t="str">
+        <x:v>核验时间</x:v>
+      </x:c>
+      <x:c r="Q2" s="10" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="24" customHeight="1">
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
+        <x:v>I-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B3" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
+      <x:c r="C3" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
         <x:v>10:00</x:v>
       </x:c>
-      <x:c r="D3" s="12" t="str">
+      <x:c r="E3" s="12" t="str">
         <x:v>11:00</x:v>
       </x:c>
-      <x:c r="E3" s="12" t="str">
+      <x:c r="F3" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="H3" s="23" t="str">
         <x:v>抵达并前往酒店</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="I3" s="23" t="str">
         <x:v>示例交通枢纽</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="J3" s="23" t="str">
         <x:v>公共交通</x:v>
       </x:c>
-      <x:c r="I3" s="23" t="str">
-        <x:v>未预订</x:v>
-      </x:c>
-      <x:c r="J3" s="23" t="n">
+      <x:c r="K3" s="23" t="str">
+        <x:v>B-001</x:v>
+      </x:c>
+      <x:c r="L3" s="23" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+      <x:c r="M3" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K3" s="23" t="str">
+      <x:c r="N3" s="23" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="L3" s="23" t="str"/>
-      <x:c r="M3" s="24" t="str">
+      <x:c r="O3" s="23" t="str">
         <x:v>虚构示例</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="P3" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="11" t="str">
+        <x:v>I-002</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B4" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
+      <x:c r="C4" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
         <x:v>14:00</x:v>
       </x:c>
-      <x:c r="D4" s="12" t="str">
+      <x:c r="E4" s="12" t="str">
         <x:v>16:00</x:v>
       </x:c>
-      <x:c r="E4" s="12" t="str">
+      <x:c r="F4" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="F4" s="23" t="str">
+      <x:c r="H4" s="23" t="str">
         <x:v>城市步行</x:v>
       </x:c>
-      <x:c r="G4" s="23" t="str">
+      <x:c r="I4" s="23" t="str">
         <x:v>示例广场</x:v>
       </x:c>
-      <x:c r="H4" s="23" t="str">
+      <x:c r="J4" s="23" t="str">
         <x:v>步行</x:v>
       </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>无需预订</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="n">
+      <x:c r="K4" s="23" t="str"/>
+      <x:c r="L4" s="23" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="M4" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K4" s="23" t="str">
+      <x:c r="N4" s="23" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="L4" s="23" t="str"/>
-      <x:c r="M4" s="24" t="str">
+      <x:c r="O4" s="23" t="str">
         <x:v>虚构示例</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="P4" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q4" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="18"/>
-      <x:c r="C5" s="15" t="str"/>
+      <x:c r="B5" s="15" t="str"/>
+      <x:c r="C5" s="18"/>
       <x:c r="D5" s="15" t="str"/>
       <x:c r="E5" s="15" t="str"/>
-      <x:c r="F5" s="25" t="str"/>
-      <x:c r="G5" s="25" t="str"/>
-      <x:c r="H5" s="25" t="str"/>
-      <x:c r="I5" s="25" t="str"/>
-      <x:c r="J5" s="25"/>
-      <x:c r="K5" s="25" t="str"/>
-      <x:c r="L5" s="25" t="str"/>
-      <x:c r="M5" s="26" t="str"/>
+      <x:c r="F5" s="15" t="str"/>
+      <x:c r="G5" s="15" t="str"/>
+      <x:c r="H5" s="26" t="str"/>
+      <x:c r="I5" s="26" t="str"/>
+      <x:c r="J5" s="26" t="str"/>
+      <x:c r="K5" s="26" t="str"/>
+      <x:c r="L5" s="26" t="str"/>
+      <x:c r="M5" s="26"/>
+      <x:c r="N5" s="26" t="str"/>
+      <x:c r="O5" s="26" t="str"/>
+      <x:c r="P5" s="27"/>
+      <x:c r="Q5" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I3:I100">
-      <x:formula1>"未预订,待确认,已确认,无需预订,已取消"</x:formula1>
+    <x:dataValidation type="list" sqref="L3:L100">
+      <x:formula1>"Planned,Ready,In progress,Done,Skipped,Blocked"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -710,93 +818,135 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>决策与协作</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
+        <x:v>Bookings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>ID</x:v>
+        <x:v>预订ID</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>提交人</x:v>
+        <x:v>类别</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>日期</x:v>
+        <x:v>供应方</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>影响日期</x:v>
+        <x:v>开始时间</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>提案</x:v>
+        <x:v>结束时间</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>原因</x:v>
+        <x:v>城市</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>状态</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>决策人</x:v>
-      </x:c>
-      <x:c r="I2" s="10" t="str">
-        <x:v>处理结果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
+        <x:v>可退</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>金额</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
+        <x:v>币种</x:v>
+      </x:c>
+      <x:c r="K2" s="9" t="str">
+        <x:v>凭证位置</x:v>
+      </x:c>
+      <x:c r="L2" s="9" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+      <x:c r="M2" s="9" t="str">
+        <x:v>核验时间</x:v>
+      </x:c>
+      <x:c r="N2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
-        <x:v>D-001</x:v>
+        <x:v>B-001</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>同行者 A</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="n">
-        <x:v>47574</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="n">
-        <x:v>47605</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>晚餐提前一小时</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>避免太晚回程</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>旅行负责人</x:v>
-      </x:c>
-      <x:c r="I3" s="24" t="str"/>
-    </x:row>
-    <x:row r="4" ht="30" customHeight="1">
+        <x:v>住宿</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>示例酒店</x:v>
+      </x:c>
+      <x:c r="D3" s="19" t="d">
+        <x:v>2030-05-01T07:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E3" s="19" t="d">
+        <x:v>2030-05-03T03:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="str">
+        <x:v>示例城</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="K3" s="23" t="str">
+        <x:v>私人档案中的预订文件夹</x:v>
+      </x:c>
+      <x:c r="L3" s="23" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+      <x:c r="M3" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="N3" s="25" t="str">
+        <x:v>不存放真实订单号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="18"/>
-      <x:c r="D4" s="18"/>
-      <x:c r="E4" s="25" t="str"/>
-      <x:c r="F4" s="25" t="str"/>
-      <x:c r="G4" s="25" t="str"/>
-      <x:c r="H4" s="25" t="str"/>
-      <x:c r="I4" s="26" t="str"/>
+      <x:c r="C4" s="15" t="str"/>
+      <x:c r="D4" s="20"/>
+      <x:c r="E4" s="20"/>
+      <x:c r="F4" s="15" t="str"/>
+      <x:c r="G4" s="15" t="str"/>
+      <x:c r="H4" s="15" t="str"/>
+      <x:c r="I4" s="15"/>
+      <x:c r="J4" s="15" t="str"/>
+      <x:c r="K4" s="26" t="str"/>
+      <x:c r="L4" s="26" t="str"/>
+      <x:c r="M4" s="27"/>
+      <x:c r="N4" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G3:G100">
-      <x:formula1>"待处理,接受,拒绝,需澄清"</x:formula1>
+      <x:formula1>"待确认,已确认,已取消,已完成"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -807,20 +957,236 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>版本记录</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
+        <x:v>Checklist</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>任务ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>类别</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>任务</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>截止日期</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>依赖</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>关联ID</x:v>
+      </x:c>
+      <x:c r="I2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>T-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>确认</x:v>
+      </x:c>
+      <x:c r="C3" s="23" t="str">
+        <x:v>出发前复核住宿</x:v>
+      </x:c>
+      <x:c r="D3" s="23" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="E3" s="29" t="d">
+        <x:v>2030-04-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str"/>
+      <x:c r="H3" s="23" t="str">
+        <x:v>B-001</x:v>
+      </x:c>
+      <x:c r="I3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="26" t="str"/>
+      <x:c r="D4" s="26" t="str"/>
+      <x:c r="E4" s="30"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F3:F100">
+      <x:formula1>"待处理,进行中,已完成,已取消,阻塞"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Preferences</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>偏好ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>范围</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>类别</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>适用人</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>偏好或约束</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>证据</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>置信度</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>生效日期</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
+        <x:v>失效日期</x:v>
+      </x:c>
+      <x:c r="K2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>P-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>本次旅行</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>节奏</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>硬约束</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="str">
+        <x:v>所有人</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>每日步行不超过虚构上限</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str">
+        <x:v>用户明确说明</x:v>
+      </x:c>
+      <x:c r="H3" s="23" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I3" s="29" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J3" s="29" t="d">
+        <x:v>2030-05-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="15" t="str"/>
+      <x:c r="D4" s="15" t="str"/>
+      <x:c r="E4" s="15" t="str"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="30"/>
+      <x:c r="J4" s="30"/>
+      <x:c r="K4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="B3:B100">
+      <x:formula1>"长期,本次旅行"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D3:D100">
+      <x:formula1>"硬约束,强偏好,一般偏好,可选"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Change Log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
         <x:v>版本</x:v>
       </x:c>
@@ -836,37 +1202,249 @@
       <x:c r="E2" s="9" t="str">
         <x:v>变更摘要</x:v>
       </x:c>
-      <x:c r="F2" s="10" t="str">
+      <x:c r="F2" s="9" t="str">
         <x:v>上一版本</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="G2" s="10" t="str">
+        <x:v>档案哈希</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B3" s="19" t="n">
-        <x:v>47574.083333333336</x:v>
+      <x:c r="B3" s="19" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
+        <x:v>M-001</x:v>
       </x:c>
       <x:c r="D3" s="23" t="str">
-        <x:v>建立草案</x:v>
+        <x:v>建立初始版本</x:v>
       </x:c>
       <x:c r="E3" s="23" t="str">
         <x:v>创建虚构示例行程</x:v>
       </x:c>
-      <x:c r="F3" s="24" t="str"/>
-    </x:row>
-    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="F3" s="23" t="str"/>
+      <x:c r="G3" s="25" t="str"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="20"/>
       <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="25" t="str"/>
-      <x:c r="E4" s="25" t="str"/>
+      <x:c r="D4" s="26" t="str"/>
+      <x:c r="E4" s="26" t="str"/>
       <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>成员ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>显示名</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>角色</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>同行关系</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>本次需求</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>权限</x:v>
+      </x:c>
+      <x:c r="G2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>旅行负责人</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D3" s="23" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="E3" s="23" t="str"/>
+      <x:c r="F3" s="23" t="str">
+        <x:v>最终确认</x:v>
+      </x:c>
+      <x:c r="G3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="11" t="str">
+        <x:v>M-002</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>同行者 A</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Member</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>同行者</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>避免太晚返程</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="str">
+        <x:v>提出意见</x:v>
+      </x:c>
+      <x:c r="G4" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="14" t="str"/>
+      <x:c r="B5" s="15" t="str"/>
+      <x:c r="C5" s="15" t="str"/>
+      <x:c r="D5" s="26" t="str"/>
+      <x:c r="E5" s="26" t="str"/>
+      <x:c r="F5" s="26" t="str"/>
+      <x:c r="G5" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C3:C100">
+      <x:formula1>"Owner,Editor,Member,Viewer"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Proposals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>提案ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>提交人</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>影响项目或日期</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>提案</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>原因</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>决策人</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>处理结果</x:v>
+      </x:c>
+      <x:c r="J2" s="10" t="str">
+        <x:v>结果版本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>PR-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>M-002</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="d">
+        <x:v>2030-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>2030-05-02</x:v>
+      </x:c>
+      <x:c r="E3" s="23" t="str">
+        <x:v>晚餐提前一小时</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>避免太晚返程</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="H3" s="23" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="I3" s="23" t="str"/>
+      <x:c r="J3" s="25" t="str"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="18"/>
+      <x:c r="D4" s="15" t="str"/>
+      <x:c r="E4" s="26" t="str"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="26" t="str"/>
+      <x:c r="J4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G3:G100">
+      <x:formula1>"待处理,接受,拒绝,需澄清"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete Travel OS lifecycle and validation (#1)
</commit_message>
<xml_diff>
--- a/templates/TravelOS-Template.xlsx
+++ b/templates/TravelOS-Template.xlsx
@@ -2,10 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旅行概览" sheetId="1" r:id="R11f90b7b6fc64149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前行程" sheetId="2" r:id="Ra898c79a5af24757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="决策与协作" sheetId="3" r:id="R4944575411664995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="4" r:id="Rce7bd37146704a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel Overview" sheetId="1" r:id="R1923f46351a44bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="2" r:id="R57f2af995ad545fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="3" r:id="R3f382a0ca7ce463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="4" r:id="Re882fef17dff4f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferences" sheetId="5" r:id="R10c94c6a9c9a44f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="6" r:id="R0d82132e5d19404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" r:id="R5b4c9e3a47264ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposals" sheetId="8" r:id="R0f4a7277c3624dd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -62,14 +66,23 @@
     </x:fill>
   </x:fills>
   <x:borders count="10">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -78,19 +91,25 @@
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
@@ -100,6 +119,7 @@
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -114,25 +134,31 @@
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:right>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -144,20 +170,25 @@
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:left>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9E2F3"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -224,13 +255,25 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -441,18 +484,20 @@
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>旅行概览</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
+        <x:v>Travel Overview</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
         <x:v>Trip ID</x:v>
       </x:c>
@@ -478,13 +523,19 @@
         <x:v>Active Version</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
+        <x:v>旅行阶段</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="J2" s="10" t="str">
+      <x:c r="K2" s="9" t="str">
+        <x:v>主时区</x:v>
+      </x:c>
+      <x:c r="L2" s="10" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="24" customHeight="1">
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
         <x:v>DEMO-001</x:v>
       </x:c>
@@ -494,29 +545,35 @@
       <x:c r="C3" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="D3" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="E3" s="17" t="n">
-        <x:v>47606</x:v>
+      <x:c r="D3" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="d">
+        <x:v>2030-05-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="F3" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
+        <x:v>M-001</x:v>
       </x:c>
       <x:c r="H3" s="21" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
       <x:c r="I3" s="12" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="J3" s="13" t="str">
+        <x:v>行前规划</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="str">
         <x:v>本行仅为虚构示例，请替换</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="24" customHeight="1">
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="15" t="str"/>
       <x:c r="C4" s="15" t="str"/>
@@ -526,11 +583,16 @@
       <x:c r="G4" s="15" t="str"/>
       <x:c r="H4" s="22" t="str"/>
       <x:c r="I4" s="15" t="str"/>
-      <x:c r="J4" s="16" t="str"/>
+      <x:c r="J4" s="15" t="str"/>
+      <x:c r="K4" s="15" t="str"/>
+      <x:c r="L4" s="16" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I3:I4">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="I3:I100">
+      <x:formula1>"行前规划,旅行中,旅行后"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J3:J100">
       <x:formula1>"Draft,Active,Completed,Cancelled"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -542,164 +604,210 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>当前行程</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
+        <x:v>Daily Plan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
+        <x:v>项目ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
         <x:v>版本</x:v>
       </x:c>
-      <x:c r="B2" s="9" t="str">
+      <x:c r="C2" s="9" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>开始</x:v>
       </x:c>
-      <x:c r="D2" s="9" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>结束</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="str">
+      <x:c r="F2" s="9" t="str">
+        <x:v>时区</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
         <x:v>城市</x:v>
       </x:c>
-      <x:c r="F2" s="9" t="str">
+      <x:c r="H2" s="9" t="str">
         <x:v>活动</x:v>
       </x:c>
-      <x:c r="G2" s="9" t="str">
+      <x:c r="I2" s="9" t="str">
         <x:v>地点</x:v>
       </x:c>
-      <x:c r="H2" s="9" t="str">
+      <x:c r="J2" s="9" t="str">
         <x:v>交通</x:v>
       </x:c>
-      <x:c r="I2" s="9" t="str">
-        <x:v>预订状态</x:v>
-      </x:c>
-      <x:c r="J2" s="9" t="str">
+      <x:c r="K2" s="9" t="str">
+        <x:v>预订ID</x:v>
+      </x:c>
+      <x:c r="L2" s="9" t="str">
+        <x:v>执行状态</x:v>
+      </x:c>
+      <x:c r="M2" s="9" t="str">
         <x:v>费用</x:v>
       </x:c>
-      <x:c r="K2" s="9" t="str">
+      <x:c r="N2" s="9" t="str">
         <x:v>币种</x:v>
       </x:c>
-      <x:c r="L2" s="9" t="str">
+      <x:c r="O2" s="9" t="str">
         <x:v>来源</x:v>
       </x:c>
-      <x:c r="M2" s="10" t="str">
+      <x:c r="P2" s="9" t="str">
+        <x:v>核验时间</x:v>
+      </x:c>
+      <x:c r="Q2" s="10" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="24" customHeight="1">
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
+        <x:v>I-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B3" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
+      <x:c r="C3" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
         <x:v>10:00</x:v>
       </x:c>
-      <x:c r="D3" s="12" t="str">
+      <x:c r="E3" s="12" t="str">
         <x:v>11:00</x:v>
       </x:c>
-      <x:c r="E3" s="12" t="str">
+      <x:c r="F3" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="F3" s="23" t="str">
+      <x:c r="H3" s="23" t="str">
         <x:v>抵达并前往酒店</x:v>
       </x:c>
-      <x:c r="G3" s="23" t="str">
+      <x:c r="I3" s="23" t="str">
         <x:v>示例交通枢纽</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
+      <x:c r="J3" s="23" t="str">
         <x:v>公共交通</x:v>
       </x:c>
-      <x:c r="I3" s="23" t="str">
-        <x:v>未预订</x:v>
-      </x:c>
-      <x:c r="J3" s="23" t="n">
+      <x:c r="K3" s="23" t="str">
+        <x:v>B-001</x:v>
+      </x:c>
+      <x:c r="L3" s="23" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+      <x:c r="M3" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K3" s="23" t="str">
+      <x:c r="N3" s="23" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="L3" s="23" t="str"/>
-      <x:c r="M3" s="24" t="str">
+      <x:c r="O3" s="23" t="str">
         <x:v>虚构示例</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="P3" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="11" t="str">
+        <x:v>I-002</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B4" s="17" t="n">
-        <x:v>47604</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
+      <x:c r="C4" s="17" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
         <x:v>14:00</x:v>
       </x:c>
-      <x:c r="D4" s="12" t="str">
+      <x:c r="E4" s="12" t="str">
         <x:v>16:00</x:v>
       </x:c>
-      <x:c r="E4" s="12" t="str">
+      <x:c r="F4" s="12" t="str">
+        <x:v>Asia/Shanghai</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
         <x:v>示例城</x:v>
       </x:c>
-      <x:c r="F4" s="23" t="str">
+      <x:c r="H4" s="23" t="str">
         <x:v>城市步行</x:v>
       </x:c>
-      <x:c r="G4" s="23" t="str">
+      <x:c r="I4" s="23" t="str">
         <x:v>示例广场</x:v>
       </x:c>
-      <x:c r="H4" s="23" t="str">
+      <x:c r="J4" s="23" t="str">
         <x:v>步行</x:v>
       </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>无需预订</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="n">
+      <x:c r="K4" s="23" t="str"/>
+      <x:c r="L4" s="23" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="M4" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K4" s="23" t="str">
+      <x:c r="N4" s="23" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="L4" s="23" t="str"/>
-      <x:c r="M4" s="24" t="str">
+      <x:c r="O4" s="23" t="str">
         <x:v>虚构示例</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="P4" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="Q4" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="14" t="str"/>
-      <x:c r="B5" s="18"/>
-      <x:c r="C5" s="15" t="str"/>
+      <x:c r="B5" s="15" t="str"/>
+      <x:c r="C5" s="18"/>
       <x:c r="D5" s="15" t="str"/>
       <x:c r="E5" s="15" t="str"/>
-      <x:c r="F5" s="25" t="str"/>
-      <x:c r="G5" s="25" t="str"/>
-      <x:c r="H5" s="25" t="str"/>
-      <x:c r="I5" s="25" t="str"/>
-      <x:c r="J5" s="25"/>
-      <x:c r="K5" s="25" t="str"/>
-      <x:c r="L5" s="25" t="str"/>
-      <x:c r="M5" s="26" t="str"/>
+      <x:c r="F5" s="15" t="str"/>
+      <x:c r="G5" s="15" t="str"/>
+      <x:c r="H5" s="26" t="str"/>
+      <x:c r="I5" s="26" t="str"/>
+      <x:c r="J5" s="26" t="str"/>
+      <x:c r="K5" s="26" t="str"/>
+      <x:c r="L5" s="26" t="str"/>
+      <x:c r="M5" s="26"/>
+      <x:c r="N5" s="26" t="str"/>
+      <x:c r="O5" s="26" t="str"/>
+      <x:c r="P5" s="27"/>
+      <x:c r="Q5" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I3:I100">
-      <x:formula1>"未预订,待确认,已确认,无需预订,已取消"</x:formula1>
+    <x:dataValidation type="list" sqref="L3:L100">
+      <x:formula1>"Planned,Ready,In progress,Done,Skipped,Blocked"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -710,93 +818,135 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>决策与协作</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
+        <x:v>Bookings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>ID</x:v>
+        <x:v>预订ID</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>提交人</x:v>
+        <x:v>类别</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>日期</x:v>
+        <x:v>供应方</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>影响日期</x:v>
+        <x:v>开始时间</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
-        <x:v>提案</x:v>
+        <x:v>结束时间</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>原因</x:v>
+        <x:v>城市</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>状态</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>决策人</x:v>
-      </x:c>
-      <x:c r="I2" s="10" t="str">
-        <x:v>处理结果</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
+        <x:v>可退</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>金额</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
+        <x:v>币种</x:v>
+      </x:c>
+      <x:c r="K2" s="9" t="str">
+        <x:v>凭证位置</x:v>
+      </x:c>
+      <x:c r="L2" s="9" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+      <x:c r="M2" s="9" t="str">
+        <x:v>核验时间</x:v>
+      </x:c>
+      <x:c r="N2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
-        <x:v>D-001</x:v>
+        <x:v>B-001</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>同行者 A</x:v>
-      </x:c>
-      <x:c r="C3" s="17" t="n">
-        <x:v>47574</x:v>
-      </x:c>
-      <x:c r="D3" s="17" t="n">
-        <x:v>47605</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:v>晚餐提前一小时</x:v>
-      </x:c>
-      <x:c r="F3" s="23" t="str">
-        <x:v>避免太晚回程</x:v>
-      </x:c>
-      <x:c r="G3" s="23" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>旅行负责人</x:v>
-      </x:c>
-      <x:c r="I3" s="24" t="str"/>
-    </x:row>
-    <x:row r="4" ht="30" customHeight="1">
+        <x:v>住宿</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>示例酒店</x:v>
+      </x:c>
+      <x:c r="D3" s="19" t="d">
+        <x:v>2030-05-01T07:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E3" s="19" t="d">
+        <x:v>2030-05-03T03:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="str">
+        <x:v>示例城</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="K3" s="23" t="str">
+        <x:v>私人档案中的预订文件夹</x:v>
+      </x:c>
+      <x:c r="L3" s="23" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+      <x:c r="M3" s="24" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="N3" s="25" t="str">
+        <x:v>不存放真实订单号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="15" t="str"/>
-      <x:c r="C4" s="18"/>
-      <x:c r="D4" s="18"/>
-      <x:c r="E4" s="25" t="str"/>
-      <x:c r="F4" s="25" t="str"/>
-      <x:c r="G4" s="25" t="str"/>
-      <x:c r="H4" s="25" t="str"/>
-      <x:c r="I4" s="26" t="str"/>
+      <x:c r="C4" s="15" t="str"/>
+      <x:c r="D4" s="20"/>
+      <x:c r="E4" s="20"/>
+      <x:c r="F4" s="15" t="str"/>
+      <x:c r="G4" s="15" t="str"/>
+      <x:c r="H4" s="15" t="str"/>
+      <x:c r="I4" s="15"/>
+      <x:c r="J4" s="15" t="str"/>
+      <x:c r="K4" s="26" t="str"/>
+      <x:c r="L4" s="26" t="str"/>
+      <x:c r="M4" s="27"/>
+      <x:c r="N4" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G3:G100">
-      <x:formula1>"待处理,接受,拒绝,需澄清"</x:formula1>
+      <x:formula1>"待确认,已确认,已取消,已完成"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -807,20 +957,236 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>版本记录</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
+        <x:v>Checklist</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>任务ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>类别</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>任务</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>截止日期</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>依赖</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>关联ID</x:v>
+      </x:c>
+      <x:c r="I2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>T-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>确认</x:v>
+      </x:c>
+      <x:c r="C3" s="23" t="str">
+        <x:v>出发前复核住宿</x:v>
+      </x:c>
+      <x:c r="D3" s="23" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="E3" s="29" t="d">
+        <x:v>2030-04-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str"/>
+      <x:c r="H3" s="23" t="str">
+        <x:v>B-001</x:v>
+      </x:c>
+      <x:c r="I3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="26" t="str"/>
+      <x:c r="D4" s="26" t="str"/>
+      <x:c r="E4" s="30"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F3:F100">
+      <x:formula1>"待处理,进行中,已完成,已取消,阻塞"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Preferences</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>偏好ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>范围</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>类别</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>适用人</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>偏好或约束</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>证据</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>置信度</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>生效日期</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
+        <x:v>失效日期</x:v>
+      </x:c>
+      <x:c r="K2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>P-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>本次旅行</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>节奏</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>硬约束</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="str">
+        <x:v>所有人</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>每日步行不超过虚构上限</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str">
+        <x:v>用户明确说明</x:v>
+      </x:c>
+      <x:c r="H3" s="23" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="I3" s="29" t="d">
+        <x:v>2030-05-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="J3" s="29" t="d">
+        <x:v>2030-05-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="K3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="15" t="str"/>
+      <x:c r="D4" s="15" t="str"/>
+      <x:c r="E4" s="15" t="str"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="30"/>
+      <x:c r="J4" s="30"/>
+      <x:c r="K4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="B3:B100">
+      <x:formula1>"长期,本次旅行"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D3:D100">
+      <x:formula1>"硬约束,强偏好,一般偏好,可选"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Change Log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
         <x:v>版本</x:v>
       </x:c>
@@ -836,37 +1202,249 @@
       <x:c r="E2" s="9" t="str">
         <x:v>变更摘要</x:v>
       </x:c>
-      <x:c r="F2" s="10" t="str">
+      <x:c r="F2" s="9" t="str">
         <x:v>上一版本</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="G2" s="10" t="str">
+        <x:v>档案哈希</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="11" t="str">
         <x:v>v0.1.0</x:v>
       </x:c>
-      <x:c r="B3" s="19" t="n">
-        <x:v>47574.083333333336</x:v>
+      <x:c r="B3" s="19" t="d">
+        <x:v>2030-04-01T02:00:00.000Z</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>旅行负责人</x:v>
+        <x:v>M-001</x:v>
       </x:c>
       <x:c r="D3" s="23" t="str">
-        <x:v>建立草案</x:v>
+        <x:v>建立初始版本</x:v>
       </x:c>
       <x:c r="E3" s="23" t="str">
         <x:v>创建虚构示例行程</x:v>
       </x:c>
-      <x:c r="F3" s="24" t="str"/>
-    </x:row>
-    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="F3" s="23" t="str"/>
+      <x:c r="G3" s="25" t="str"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str"/>
       <x:c r="B4" s="20"/>
       <x:c r="C4" s="15" t="str"/>
-      <x:c r="D4" s="25" t="str"/>
-      <x:c r="E4" s="25" t="str"/>
+      <x:c r="D4" s="26" t="str"/>
+      <x:c r="E4" s="26" t="str"/>
       <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>成员ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>显示名</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>角色</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>同行关系</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>本次需求</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>权限</x:v>
+      </x:c>
+      <x:c r="G2" s="10" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>旅行负责人</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D3" s="23" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="E3" s="23" t="str"/>
+      <x:c r="F3" s="23" t="str">
+        <x:v>最终确认</x:v>
+      </x:c>
+      <x:c r="G3" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="11" t="str">
+        <x:v>M-002</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>同行者 A</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Member</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>同行者</x:v>
+      </x:c>
+      <x:c r="E4" s="23" t="str">
+        <x:v>避免太晚返程</x:v>
+      </x:c>
+      <x:c r="F4" s="23" t="str">
+        <x:v>提出意见</x:v>
+      </x:c>
+      <x:c r="G4" s="25" t="str">
+        <x:v>虚构示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="14" t="str"/>
+      <x:c r="B5" s="15" t="str"/>
+      <x:c r="C5" s="15" t="str"/>
+      <x:c r="D5" s="26" t="str"/>
+      <x:c r="E5" s="26" t="str"/>
+      <x:c r="F5" s="26" t="str"/>
+      <x:c r="G5" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C3:C100">
+      <x:formula1>"Owner,Editor,Member,Viewer"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Proposals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>提案ID</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>提交人</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>影响项目或日期</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>提案</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>原因</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>决策人</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:v>处理结果</x:v>
+      </x:c>
+      <x:c r="J2" s="10" t="str">
+        <x:v>结果版本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>PR-001</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>M-002</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="d">
+        <x:v>2030-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>2030-05-02</x:v>
+      </x:c>
+      <x:c r="E3" s="23" t="str">
+        <x:v>晚餐提前一小时</x:v>
+      </x:c>
+      <x:c r="F3" s="23" t="str">
+        <x:v>避免太晚返程</x:v>
+      </x:c>
+      <x:c r="G3" s="23" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="H3" s="23" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="I3" s="23" t="str"/>
+      <x:c r="J3" s="25" t="str"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="14" t="str"/>
+      <x:c r="B4" s="15" t="str"/>
+      <x:c r="C4" s="18"/>
+      <x:c r="D4" s="15" t="str"/>
+      <x:c r="E4" s="26" t="str"/>
+      <x:c r="F4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str"/>
+      <x:c r="H4" s="26" t="str"/>
+      <x:c r="I4" s="26" t="str"/>
+      <x:c r="J4" s="28" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G3:G100">
+      <x:formula1>"待处理,接受,拒绝,需澄清"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>